<commit_message>
Sync published toolbox with current scGEAToolbox_dev build
Regenerated by copyDepsWithStructure. Drops files removed from dev
(external/ml_umap45, fun_alona_subtypes, @SingleCellExperiment2, etc.),
the demo example data no longer shipped, and ml_scDock dev clutter
(dock_output, PDFs, .claude).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/PanglaoDB/cellsubtypes.xlsx
+++ b/assets/PanglaoDB/cellsubtypes.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="libxl" lastEdited="7" lowestEdited="7" rupBuild="4.6.0"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449A1452-B806-4609-8D8E-B2F725814F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3525" yWindow="2130" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3525" yWindow="2130" windowWidth="21600" windowHeight="11235"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="358" uniqueCount="247">
   <si>
     <t>PositiveMarkers</t>
   </si>
@@ -730,13 +730,49 @@
   </si>
   <si>
     <t>Glutamatergic</t>
+  </si>
+  <si>
+    <t>Thymocytes</t>
+  </si>
+  <si>
+    <t>Neural stem/precursor</t>
+  </si>
+  <si>
+    <t>Neuroblasts</t>
+  </si>
+  <si>
+    <t>Neuroendocrine</t>
+  </si>
+  <si>
+    <t>NOTCH1,CD38,CXCR4,TNF,CD2,CD4,CD5,CD8A,IL2RA,CD69,SLAMF1,TAGAP,MS4A4B,UCP2,TSHR,CD27,CD28,BCL6,CIDEA,EZR</t>
+  </si>
+  <si>
+    <t>SOX1,PROM1,IGF1R,SP8,GFAP,RBM3,SOX3,S100B,SLC1A3,NEUROD4,NEUROG1,NEUROG2,NHLH1,PPP1R17,TMTC4,EOMES,PLEKHH2,TLR3,PARP12,P2RX7,INAFM2,ISG15,IGFBP3,IFIT1,IFI44,MGAT5,PBK,DLX2,CBX3,RND3,DLX5,SP9,POU3F4,DYNLT1C,BARHL2,LHX9,SHOX2,DBX1,DLL3,PITX2,OTX1,ARX,NXPH1,TOX3,ASCL2,HES5,HOPX,NEUROD1,PRSS56,SOX9,ALDOC,APOE,ID4,SOX2,DCX,CCND2,DLX1,S100A6</t>
+  </si>
+  <si>
+    <t>NTNG1,TSHZ1,SP9,SP8,PROK2,ASCL1,DLL3,SALL3,DRAXIN,ERBB4,TRIM32,IGFBPL1,EOMES,PBX1,CUX2,ISL1,PHF1,NEUROG1,NKX6-1,NEUROG2,MAPK7,PROKR2,POU6F2,ITGA6,EFNA2,DCX,CCKAR,CCKBR,GRM5,EZH2,DLX2,MARK2,LRP8,VLDLR,DAB1,NCAN,EPHA4,TACC3,EGFR,TUBB3,SIRT1,NCAM1,NEUROD1,SCGN,NES,WT1,ZBED4,PROS1,CNR1</t>
+  </si>
+  <si>
+    <t>PPP1R1B,CLASP2,MKL2,FXYD7,DPF1,PENK,GRM5,SFXN5,TAC1,CCDC85C,ATXN1,GPR88,PDE10A,SST,CXCL14,NPY,NRGN,SCN2B,ABHD2,SPOCK1,NEGR1,DUSP26,ARHGDIG,CCK,PRSS12,SERPINI1,NKX2-2</t>
+  </si>
+  <si>
+    <t>immature T cells of the thymus</t>
+  </si>
+  <si>
+    <t>progenitors rather than mature neurons</t>
+  </si>
+  <si>
+    <t>committed neuronal progenitors</t>
+  </si>
+  <si>
+    <t>a distinct lineage, grouped under Neurons in the source list</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -777,7 +813,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -785,16 +821,18 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -815,7 +853,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -932,7 +970,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -956,9 +994,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -982,7 +1020,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1017,7 +1055,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1035,7 +1073,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1060,7 +1098,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1076,19 +1114,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F84"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F88"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="1367.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="73.28515625" customWidth="1"/>
-    <col min="6" max="6" width="97.28515625" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="true"/>
+    <col min="2" max="2" width="22.7109375" customWidth="true"/>
+    <col min="3" max="3" width="1367.140625" style="1" customWidth="true"/>
+    <col min="4" max="4" width="16.28515625" style="2" customWidth="true"/>
+    <col min="5" max="5" width="73.28515625" customWidth="true"/>
+    <col min="6" max="6" width="97.28515625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1108,7 +1146,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1119,7 +1157,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1130,7 +1168,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1144,7 +1182,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1158,7 +1196,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1175,7 +1213,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1189,7 +1227,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1203,7 +1241,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1214,7 +1252,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1225,7 +1263,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1236,7 +1274,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1247,7 +1285,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1258,7 +1296,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1269,7 +1307,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1280,7 +1318,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -1291,7 +1329,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -1302,7 +1340,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1313,7 +1351,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -1324,7 +1362,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -1335,7 +1373,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -1346,7 +1384,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -1357,7 +1395,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -1368,7 +1406,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1379,7 +1417,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -1390,7 +1428,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -1401,7 +1439,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1412,7 +1450,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1429,7 +1467,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>37</v>
       </c>
@@ -1440,7 +1478,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -1451,7 +1489,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -1468,7 +1506,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1485,7 +1523,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1502,7 +1540,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1519,7 +1557,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -1533,7 +1571,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -1547,7 +1585,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -1561,7 +1599,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -1575,7 +1613,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1592,7 +1630,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>37</v>
       </c>
@@ -1609,7 +1647,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>87</v>
       </c>
@@ -1623,7 +1661,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>87</v>
       </c>
@@ -1637,7 +1675,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>87</v>
       </c>
@@ -1651,7 +1689,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -1668,7 +1706,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>87</v>
       </c>
@@ -1682,7 +1720,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>87</v>
       </c>
@@ -1696,7 +1734,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>88</v>
       </c>
@@ -1713,7 +1751,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -1730,7 +1768,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>88</v>
       </c>
@@ -1747,7 +1785,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>88</v>
       </c>
@@ -1761,7 +1799,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>89</v>
       </c>
@@ -1778,7 +1816,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>89</v>
       </c>
@@ -1795,7 +1833,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>89</v>
       </c>
@@ -1812,7 +1850,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>90</v>
       </c>
@@ -1826,7 +1864,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="55" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>90</v>
       </c>
@@ -1840,7 +1878,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="56" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>90</v>
       </c>
@@ -1857,7 +1895,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="57" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>90</v>
       </c>
@@ -1871,7 +1909,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="58" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>90</v>
       </c>
@@ -1888,7 +1926,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="59" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>91</v>
       </c>
@@ -1902,7 +1940,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="60" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>91</v>
       </c>
@@ -1919,7 +1957,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="61" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>91</v>
       </c>
@@ -1933,7 +1971,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="62" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>92</v>
       </c>
@@ -1950,7 +1988,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="63" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>92</v>
       </c>
@@ -1967,7 +2005,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="64" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>92</v>
       </c>
@@ -1984,7 +2022,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="65" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>92</v>
       </c>
@@ -2001,7 +2039,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="66" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>93</v>
       </c>
@@ -2015,7 +2053,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="67" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>93</v>
       </c>
@@ -2029,7 +2067,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="68" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>93</v>
       </c>
@@ -2043,7 +2081,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="69" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>93</v>
       </c>
@@ -2057,7 +2095,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="70" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>93</v>
       </c>
@@ -2074,7 +2112,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="71" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>94</v>
       </c>
@@ -2088,7 +2126,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="72" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>94</v>
       </c>
@@ -2102,7 +2140,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="73" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>94</v>
       </c>
@@ -2116,7 +2154,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="74" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>94</v>
       </c>
@@ -2130,7 +2168,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="75" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>95</v>
       </c>
@@ -2147,7 +2185,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="76" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>95</v>
       </c>
@@ -2164,7 +2202,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="77" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>95</v>
       </c>
@@ -2178,7 +2216,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="78" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>96</v>
       </c>
@@ -2192,7 +2230,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="79" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>96</v>
       </c>
@@ -2209,7 +2247,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="80" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>96</v>
       </c>
@@ -2223,7 +2261,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="81" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>96</v>
       </c>
@@ -2237,7 +2275,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="82" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>97</v>
       </c>
@@ -2254,7 +2292,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="83" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>97</v>
       </c>
@@ -2268,7 +2306,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="84" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>97</v>
       </c>
@@ -2280,6 +2318,70 @@
       </c>
       <c r="E84" t="s">
         <v>213</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="B85" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D85" s="2"/>
+      <c r="E85" s="0"/>
+      <c r="F85" s="0" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B86" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="D86" s="2"/>
+      <c r="E86" s="0"/>
+      <c r="F86" s="0" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B87" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D87" s="2"/>
+      <c r="E87" s="0"/>
+      <c r="F87" s="0" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B88" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D88" s="2"/>
+      <c r="E88" s="0"/>
+      <c r="F88" s="0" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>